<commit_message>
[NEW] Update character actions
</commit_message>
<xml_diff>
--- a/VNFramework/Assets/Resources/story/Test.xlsx
+++ b/VNFramework/Assets/Resources/story/Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angel\Desktop\VNFramework\Assets\Resources\story\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E36A411-CA8F-4609-BEF0-711E484007A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1D53A43-C067-4EE4-9A85-D24F3C5A1B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,16 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="21">
   <si>
     <t>Annie</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Hi!</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Bella</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -56,6 +52,62 @@
   </si>
   <si>
     <t>Bye!</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Name</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dialogue</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Avatar</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vocal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BGImage</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BGM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hi! Long long long long long long Intro</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>appearAt(x,y)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>moveTo(x,y)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>disappear</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Character1Action</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Character1Image</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Character2Action</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Character2Image</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -381,79 +433,160 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="58" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="21" customWidth="1"/>
+    <col min="10" max="10" width="15.21875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="43.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="G3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C4" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="G4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" t="s">
+        <v>0</v>
+      </c>
+      <c r="I4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" t="s">
         <v>5</v>
       </c>
-      <c r="C4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C6" t="s">
+        <v>0</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" t="s">
         <v>6</v>
       </c>
-      <c r="C5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
-        <v>0</v>
+      <c r="C7" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[NEW] Update DOTween and choices
</commit_message>
<xml_diff>
--- a/VNFramework/Assets/Resources/story/Test.xlsx
+++ b/VNFramework/Assets/Resources/story/Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angel\Desktop\VNFramework\Assets\Resources\story\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1D53A43-C067-4EE4-9A85-D24F3C5A1B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25D247E4-5B77-4855-9E4E-2967B7B44ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
   <si>
     <t>Annie</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -108,6 +108,34 @@
   </si>
   <si>
     <t>Character2Image</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>X1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>X2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>choice</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>choice1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>choice2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Test</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Test2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -433,17 +461,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="58" customWidth="1"/>
-    <col min="7" max="7" width="15.88671875" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="21" customWidth="1"/>
-    <col min="10" max="10" width="15.21875" customWidth="1"/>
+    <col min="7" max="8" width="15.88671875" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="11" width="21" customWidth="1"/>
+    <col min="12" max="12" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -466,16 +494,22 @@
         <v>17</v>
       </c>
       <c r="H1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" t="s">
         <v>18</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>19</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
+        <v>22</v>
+      </c>
+      <c r="L1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="43.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="43.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -497,11 +531,14 @@
       <c r="G2" t="s">
         <v>14</v>
       </c>
-      <c r="H2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -517,14 +554,17 @@
       <c r="G3" t="s">
         <v>16</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>14</v>
       </c>
-      <c r="J3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -540,14 +580,20 @@
       <c r="G4" t="s">
         <v>14</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4">
         <v>0</v>
       </c>
       <c r="I4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J4" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K4">
+        <v>-540</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -560,8 +606,11 @@
       <c r="G5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H5">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -571,11 +620,11 @@
       <c r="C6" t="s">
         <v>0</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -587,6 +636,23 @@
       </c>
       <c r="G7" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[NEW] Update Load and fix bug with audio playing
</commit_message>
<xml_diff>
--- a/VNFramework/Assets/Resources/story/Test.xlsx
+++ b/VNFramework/Assets/Resources/story/Test.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11460"/>
+    <workbookView windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="32">
   <si>
     <t>Name</t>
   </si>
@@ -63,6 +63,18 @@
   </si>
   <si>
     <t>Character2Image</t>
+  </si>
+  <si>
+    <t>LastBGImage</t>
+  </si>
+  <si>
+    <t>LastBGM</t>
+  </si>
+  <si>
+    <t>LastX1</t>
+  </si>
+  <si>
+    <t>LastX2</t>
   </si>
   <si>
     <t>Annie</t>
@@ -123,14 +135,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -586,148 +591,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1052,17 +1057,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="58" customWidth="1"/>
-    <col min="7" max="8" width="15.8857142857143" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="11" width="21" customWidth="1"/>
-    <col min="12" max="12" width="15.2190476190476" customWidth="1"/>
+    <col min="2" max="2" width="39.2857142857143" customWidth="1"/>
+    <col min="6" max="6" width="6.14285714285714" customWidth="1"/>
+    <col min="7" max="7" width="12.1428571428571" customWidth="1"/>
+    <col min="8" max="8" width="8.57142857142857" customWidth="1"/>
+    <col min="9" max="9" width="11.7142857142857" customWidth="1"/>
+    <col min="10" max="10" width="13.2857142857143" customWidth="1"/>
+    <col min="11" max="11" width="7.57142857142857" customWidth="1"/>
+    <col min="12" max="12" width="10.1428571428571" customWidth="1"/>
+    <col min="13" max="13" width="11.1428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:16">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1099,16 +1108,28 @@
       <c r="L1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" ht="43.8" customHeight="1" spans="1:9">
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" ht="17" customHeight="1" spans="1:16">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1120,318 +1141,808 @@
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>-900</v>
       </c>
       <c r="I2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>16</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2">
+        <v>1</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>21</v>
+      </c>
+      <c r="I3" t="s">
+        <v>16</v>
       </c>
       <c r="J3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="L3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
+        <v>19</v>
+      </c>
+      <c r="M3">
+        <f>IF(E2&lt;&gt;"",E2,M2)</f>
+        <v>1</v>
+      </c>
+      <c r="N3">
+        <f>IF(F2&lt;&gt;"",F2,N2)</f>
+        <v>1</v>
+      </c>
+      <c r="O3">
+        <f>IF(H2&lt;&gt;"",H2,O2)</f>
+        <v>-900</v>
+      </c>
+      <c r="P3">
+        <f>IF(K2&lt;&gt;"",K2,P2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E4">
         <v>3</v>
       </c>
       <c r="G4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>-840</v>
       </c>
       <c r="I4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J4" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="K4">
-        <v>-540</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="L4" t="s">
+        <v>19</v>
+      </c>
+      <c r="M4">
+        <f t="shared" ref="M4:M24" si="0">IF(E3&lt;&gt;"",E3,M3)</f>
+        <v>1</v>
+      </c>
+      <c r="N4">
+        <f t="shared" ref="N4:N24" si="1">IF(F3&lt;&gt;"",F3,N3)</f>
+        <v>1</v>
+      </c>
+      <c r="O4">
+        <f t="shared" ref="O4:O24" si="2">IF(H3&lt;&gt;"",H3,O3)</f>
+        <v>-900</v>
+      </c>
+      <c r="P4">
+        <f t="shared" ref="P4:P24" si="3">IF(K3&lt;&gt;"",K3,P3)</f>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G5" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="H5">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+      <c r="L5" t="s">
+        <v>19</v>
+      </c>
+      <c r="M5">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O5">
+        <f t="shared" si="2"/>
+        <v>-840</v>
+      </c>
+      <c r="P5">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" t="s">
         <v>21</v>
       </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
-      <c r="J6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="L6" t="s">
+        <v>19</v>
+      </c>
+      <c r="M6">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O6">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" t="s">
+        <v>16</v>
+      </c>
+      <c r="M7">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O7">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
         <v>22</v>
       </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="M8">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N8">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" t="s">
         <v>18</v>
       </c>
-      <c r="C8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
+      <c r="H9">
+        <v>100</v>
+      </c>
+      <c r="I9" t="s">
+        <v>16</v>
+      </c>
+      <c r="M9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="N9">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O9">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
+        <v>16</v>
+      </c>
+      <c r="I10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M10">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="N10">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O10">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="P10">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" t="s">
+        <v>18</v>
+      </c>
+      <c r="K11">
+        <v>240</v>
+      </c>
+      <c r="L11" t="s">
+        <v>19</v>
+      </c>
+      <c r="M11">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="N11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O11">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="P11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" t="s">
         <v>22</v>
       </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" t="s">
-        <v>18</v>
-      </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E12">
         <v>3</v>
       </c>
-    </row>
-    <row r="13" spans="1:3">
+      <c r="I12" t="s">
+        <v>16</v>
+      </c>
+      <c r="L12" t="s">
+        <v>19</v>
+      </c>
+      <c r="M12">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="N12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O12">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="P12">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
+        <v>19</v>
+      </c>
+      <c r="G13" t="s">
+        <v>23</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13" t="s">
+        <v>16</v>
+      </c>
+      <c r="L13" t="s">
+        <v>19</v>
+      </c>
+      <c r="M13">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N13">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O13">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="P13">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" t="s">
+        <v>16</v>
+      </c>
+      <c r="I14" t="s">
+        <v>16</v>
+      </c>
+      <c r="L14" t="s">
+        <v>19</v>
+      </c>
+      <c r="M14">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N14">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P14">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" t="s">
+        <v>16</v>
+      </c>
+      <c r="L15" t="s">
+        <v>19</v>
+      </c>
+      <c r="M15">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O15">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P15">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="I16" t="s">
+        <v>16</v>
+      </c>
+      <c r="L16" t="s">
+        <v>19</v>
+      </c>
+      <c r="M16">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N16">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P16">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" t="s">
+        <v>19</v>
+      </c>
+      <c r="G17" t="s">
         <v>21</v>
       </c>
-      <c r="C14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="I17" t="s">
+        <v>16</v>
+      </c>
+      <c r="L17" t="s">
+        <v>19</v>
+      </c>
+      <c r="M17">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="N17">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" t="s">
+        <v>16</v>
+      </c>
+      <c r="L18" t="s">
+        <v>19</v>
+      </c>
+      <c r="M18">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="N18">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O18">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16">
+      <c r="A19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" t="s">
+        <v>16</v>
+      </c>
+      <c r="L19" t="s">
+        <v>19</v>
+      </c>
+      <c r="M19">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="N19">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16">
+      <c r="A20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" t="s">
         <v>22</v>
       </c>
-      <c r="C15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" t="s">
-        <v>12</v>
-      </c>
-      <c r="E16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17" t="s">
-        <v>20</v>
-      </c>
-      <c r="C17" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B18" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>12</v>
-      </c>
-      <c r="B19" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" t="s">
-        <v>12</v>
-      </c>
-      <c r="B20" t="s">
-        <v>18</v>
-      </c>
       <c r="C20" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E20">
         <v>3</v>
       </c>
-    </row>
-    <row r="21" spans="1:3">
+      <c r="G20" t="s">
+        <v>18</v>
+      </c>
+      <c r="H20">
+        <v>540</v>
+      </c>
+      <c r="I20" t="s">
+        <v>16</v>
+      </c>
+      <c r="L20" t="s">
+        <v>19</v>
+      </c>
+      <c r="M20">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="N20">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O20">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P20">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16">
       <c r="A21" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C21" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
+        <v>19</v>
+      </c>
+      <c r="I21" t="s">
+        <v>16</v>
+      </c>
+      <c r="L21" t="s">
+        <v>19</v>
+      </c>
+      <c r="M21">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N21">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O21">
+        <f t="shared" si="2"/>
+        <v>540</v>
+      </c>
+      <c r="P21">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16">
       <c r="A22" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B22" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C22" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
+        <v>16</v>
+      </c>
+      <c r="I22" t="s">
+        <v>16</v>
+      </c>
+      <c r="L22" t="s">
+        <v>19</v>
+      </c>
+      <c r="M22">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N22">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O22">
+        <f t="shared" si="2"/>
+        <v>540</v>
+      </c>
+      <c r="P22">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16">
       <c r="A23" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C23" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5">
+        <v>16</v>
+      </c>
+      <c r="I23" t="s">
+        <v>16</v>
+      </c>
+      <c r="L23" t="s">
+        <v>19</v>
+      </c>
+      <c r="M23">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N23">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O23">
+        <f t="shared" si="2"/>
+        <v>540</v>
+      </c>
+      <c r="P23">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B24" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C24" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D24" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E24" t="s">
-        <v>27</v>
+        <v>31</v>
+      </c>
+      <c r="M24">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N24">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="O24">
+        <f t="shared" si="2"/>
+        <v>540</v>
+      </c>
+      <c r="P24">
+        <f t="shared" si="3"/>
+        <v>240</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[NEW] Update history and fix menu panel bugs
</commit_message>
<xml_diff>
--- a/VNFramework/Assets/Resources/story/Test.xlsx
+++ b/VNFramework/Assets/Resources/story/Test.xlsx
@@ -1144,7 +1144,7 @@
         <v>18</v>
       </c>
       <c r="H2">
-        <v>-900</v>
+        <v>0</v>
       </c>
       <c r="I2" t="s">
         <v>16</v>
@@ -1185,7 +1185,7 @@
         <v>18</v>
       </c>
       <c r="K3">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="L3" t="s">
         <v>19</v>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="O3">
         <f>IF(H2&lt;&gt;"",H2,O2)</f>
-        <v>-900</v>
+        <v>0</v>
       </c>
       <c r="P3">
         <f>IF(K2&lt;&gt;"",K2,P2)</f>
@@ -1224,7 +1224,7 @@
         <v>18</v>
       </c>
       <c r="H4">
-        <v>-840</v>
+        <v>0</v>
       </c>
       <c r="I4" t="s">
         <v>16</v>
@@ -1233,7 +1233,7 @@
         <v>23</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>-540</v>
       </c>
       <c r="L4" t="s">
         <v>19</v>
@@ -1248,11 +1248,11 @@
       </c>
       <c r="O4">
         <f t="shared" ref="O4:O24" si="2">IF(H3&lt;&gt;"",H3,O3)</f>
-        <v>-900</v>
+        <v>0</v>
       </c>
       <c r="P4">
         <f t="shared" ref="P4:P24" si="3">IF(K3&lt;&gt;"",K3,P3)</f>
-        <v>900</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:16">
@@ -1269,7 +1269,7 @@
         <v>23</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="I5" t="s">
         <v>16</v>
@@ -1287,11 +1287,11 @@
       </c>
       <c r="O5">
         <f t="shared" si="2"/>
-        <v>-840</v>
+        <v>0</v>
       </c>
       <c r="P5">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-540</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -1323,11 +1323,11 @@
       </c>
       <c r="O6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="P6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-540</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -1356,11 +1356,11 @@
       </c>
       <c r="O7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="P7">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-540</v>
       </c>
     </row>
     <row r="8" spans="1:16">
@@ -1386,11 +1386,11 @@
       </c>
       <c r="O8">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="P8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-540</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -1422,11 +1422,11 @@
       </c>
       <c r="O9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="P9">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-540</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="P10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-540</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="P11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-540</v>
       </c>
     </row>
     <row r="12" spans="1:16">

</xml_diff>

<commit_message>
[NEW] Update input name, goto function and gallery
</commit_message>
<xml_diff>
--- a/VNFramework/Assets/Resources/story/Test.xlsx
+++ b/VNFramework/Assets/Resources/story/Test.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="33">
   <si>
     <t>Name</t>
   </si>
@@ -80,49 +80,52 @@
     <t>Annie</t>
   </si>
   <si>
-    <t>Hi! Long long long long long long Intro</t>
+    <t>Hi [Name]! Long long long long long long Intro</t>
   </si>
   <si>
     <t>appearAt(x,y)</t>
   </si>
   <si>
+    <t>[Name]</t>
+  </si>
+  <si>
+    <t>Hello!</t>
+  </si>
+  <si>
     <t>Bella</t>
   </si>
   <si>
-    <t>Hello!</t>
-  </si>
-  <si>
     <t>disappear</t>
   </si>
   <si>
+    <t>How you doing [Name]?</t>
+  </si>
+  <si>
+    <t>moveTo(x,y)</t>
+  </si>
+  <si>
+    <t>Fine ty and U?</t>
+  </si>
+  <si>
+    <t>Not bad</t>
+  </si>
+  <si>
+    <t>Bye!</t>
+  </si>
+  <si>
     <t>How you doing?</t>
   </si>
   <si>
-    <t>moveTo(x,y)</t>
-  </si>
-  <si>
-    <t>Fine ty and U?</t>
-  </si>
-  <si>
-    <t>Not bad</t>
-  </si>
-  <si>
-    <t>Bye!</t>
+    <t>Bye [Name]!</t>
   </si>
   <si>
     <t>choice</t>
   </si>
   <si>
-    <t>choice1</t>
-  </si>
-  <si>
-    <t>Test</t>
-  </si>
-  <si>
-    <t>choice2</t>
-  </si>
-  <si>
     <t>Test2</t>
+  </si>
+  <si>
+    <t>Test3</t>
   </si>
 </sst>
 </file>
@@ -1170,13 +1173,13 @@
         <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
       <c r="G3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I3" t="s">
         <v>16</v>
@@ -1188,7 +1191,7 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M3">
         <f>IF(E2&lt;&gt;"",E2,M2)</f>
@@ -1212,7 +1215,7 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
         <v>16</v>
@@ -1230,13 +1233,13 @@
         <v>16</v>
       </c>
       <c r="J4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K4">
         <v>-540</v>
       </c>
       <c r="L4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M4">
         <f t="shared" ref="M4:M24" si="0">IF(E3&lt;&gt;"",E3,M3)</f>
@@ -1260,13 +1263,13 @@
         <v>19</v>
       </c>
       <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" t="s">
         <v>24</v>
-      </c>
-      <c r="C5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G5" t="s">
-        <v>23</v>
       </c>
       <c r="H5">
         <v>540</v>
@@ -1275,7 +1278,7 @@
         <v>16</v>
       </c>
       <c r="L5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M5">
         <f t="shared" si="0"/>
@@ -1299,7 +1302,7 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
         <v>16</v>
@@ -1308,10 +1311,10 @@
         <v>16</v>
       </c>
       <c r="J6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M6">
         <f t="shared" si="0"/>
@@ -1335,13 +1338,13 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
         <v>16</v>
       </c>
       <c r="G7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I7" t="s">
         <v>16</v>
@@ -1368,7 +1371,7 @@
         <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
         <v>16</v>
@@ -1398,10 +1401,10 @@
         <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G9" t="s">
         <v>18</v>
@@ -1434,7 +1437,7 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C10" t="s">
         <v>16</v>
@@ -1464,7 +1467,7 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
         <v>16</v>
@@ -1479,7 +1482,7 @@
         <v>240</v>
       </c>
       <c r="L11" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M11">
         <f t="shared" si="0"/>
@@ -1503,7 +1506,7 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
         <v>16</v>
@@ -1515,7 +1518,7 @@
         <v>16</v>
       </c>
       <c r="L12" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M12">
         <f t="shared" si="0"/>
@@ -1539,13 +1542,13 @@
         <v>19</v>
       </c>
       <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G13" t="s">
         <v>24</v>
-      </c>
-      <c r="C13" t="s">
-        <v>19</v>
-      </c>
-      <c r="G13" t="s">
-        <v>23</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -1554,7 +1557,7 @@
         <v>16</v>
       </c>
       <c r="L13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M13">
         <f t="shared" si="0"/>
@@ -1578,7 +1581,7 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C14" t="s">
         <v>16</v>
@@ -1587,7 +1590,7 @@
         <v>16</v>
       </c>
       <c r="L14" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M14">
         <f t="shared" si="0"/>
@@ -1611,7 +1614,7 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C15" t="s">
         <v>16</v>
@@ -1620,7 +1623,7 @@
         <v>16</v>
       </c>
       <c r="L15" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M15">
         <f t="shared" si="0"/>
@@ -1644,7 +1647,7 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C16" t="s">
         <v>16</v>
@@ -1656,7 +1659,7 @@
         <v>16</v>
       </c>
       <c r="L16" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M16">
         <f t="shared" si="0"/>
@@ -1680,19 +1683,19 @@
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C17" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G17" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I17" t="s">
         <v>16</v>
       </c>
       <c r="L17" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M17">
         <f t="shared" si="0"/>
@@ -1716,13 +1719,13 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C18" t="s">
         <v>16</v>
       </c>
       <c r="L18" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M18">
         <f t="shared" si="0"/>
@@ -1746,13 +1749,13 @@
         <v>16</v>
       </c>
       <c r="B19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C19" t="s">
         <v>16</v>
       </c>
       <c r="L19" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M19">
         <f t="shared" si="0"/>
@@ -1776,7 +1779,7 @@
         <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C20" t="s">
         <v>16</v>
@@ -1794,7 +1797,7 @@
         <v>16</v>
       </c>
       <c r="L20" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M20">
         <f t="shared" si="0"/>
@@ -1818,16 +1821,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C21" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I21" t="s">
         <v>16</v>
       </c>
       <c r="L21" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M21">
         <f t="shared" si="0"/>
@@ -1851,7 +1854,7 @@
         <v>16</v>
       </c>
       <c r="B22" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C22" t="s">
         <v>16</v>
@@ -1860,7 +1863,7 @@
         <v>16</v>
       </c>
       <c r="L22" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M22">
         <f t="shared" si="0"/>
@@ -1884,7 +1887,7 @@
         <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C23" t="s">
         <v>16</v>
@@ -1893,7 +1896,7 @@
         <v>16</v>
       </c>
       <c r="L23" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M23">
         <f t="shared" si="0"/>
@@ -1914,19 +1917,19 @@
     </row>
     <row r="24" spans="1:16">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C24" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D24" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E24" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M24">
         <f t="shared" si="0"/>

</xml_diff>